<commit_message>
move to external .json file like a sane person
</commit_message>
<xml_diff>
--- a/Project List.xlsx
+++ b/Project List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\conno\Documents\UNI\PAST\Project Work\PASTdle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9C6C52B-17E7-437B-AC29-940FAEC19A9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46871AA3-6E55-45C4-93F3-66DCF2EB10A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{05053F43-13BA-4F95-AF36-FFC7FBE442FD}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="165">
   <si>
     <t>ID</t>
   </si>
@@ -399,13 +399,158 @@
   </si>
   <si>
     <t>Active?</t>
+  </si>
+  <si>
+    <t>WEBSITE</t>
+  </si>
+  <si>
+    <t>PAST Website</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>BSHP</t>
+  </si>
+  <si>
+    <t>BinarX School Holidary Program</t>
+  </si>
+  <si>
+    <t>POLO</t>
+  </si>
+  <si>
+    <t>PAST Team Shirts</t>
+  </si>
+  <si>
+    <t>outreach, binar, binarx</t>
+  </si>
+  <si>
+    <t>flatsat, mission</t>
+  </si>
+  <si>
+    <t>cubesat, mission</t>
+  </si>
+  <si>
+    <t>manufacturing, coil</t>
+  </si>
+  <si>
+    <t>test</t>
+  </si>
+  <si>
+    <t>test, integration, board</t>
+  </si>
+  <si>
+    <t>test, integration</t>
+  </si>
+  <si>
+    <t>magnetic, test, integration</t>
+  </si>
+  <si>
+    <t>sun, test, cubesat</t>
+  </si>
+  <si>
+    <t>dashboard</t>
+  </si>
+  <si>
+    <t>c2s, cubesat, camera, payload</t>
+  </si>
+  <si>
+    <t>hab, high altitude, balloon</t>
+  </si>
+  <si>
+    <t>hab, high altitude, balloon, comms, starcomm</t>
+  </si>
+  <si>
+    <t>hab, high altitude, balloon, starcomm</t>
+  </si>
+  <si>
+    <t>legacy</t>
+  </si>
+  <si>
+    <t>computer, cubesat</t>
+  </si>
+  <si>
+    <t>comms, starcomm, handheld</t>
+  </si>
+  <si>
+    <t>comms, starcomm, cubesat</t>
+  </si>
+  <si>
+    <t>comms, starcomm</t>
+  </si>
+  <si>
+    <t>eps, test</t>
+  </si>
+  <si>
+    <t>eps, test, cubesat</t>
+  </si>
+  <si>
+    <t>eps, legacy</t>
+  </si>
+  <si>
+    <t>eps, cubesat</t>
+  </si>
+  <si>
+    <t>discord, bot</t>
+  </si>
+  <si>
+    <t>cubesat, starcomm, comms</t>
+  </si>
+  <si>
+    <t>cubesat, structure</t>
+  </si>
+  <si>
+    <t>hab, chassis, balloon, structure</t>
+  </si>
+  <si>
+    <t>eps</t>
+  </si>
+  <si>
+    <t>outreach, marketing</t>
+  </si>
+  <si>
+    <t>The coil winder is an ongoing project to develop hardware and processes to manufacture our own custom wire coils. This has applications in cubesat control and actuator system development, and is a critical part of developing our own custom control hardware.</t>
+  </si>
+  <si>
+    <t>The Cubesat Camera System is an ongoing project to develop an in-house low-cost earth imaging system for a 1U cubesat. C2S is the primary payload for the upcoming CubeSat being developed by PAST.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The PAST discord bot is an ongoing project to develop automation tools for our primary communication and data channels, including the PAST discord. </t>
+  </si>
+  <si>
+    <r>
+      <t>The BinarX school holiday program was a five-day outreach event hosted in January 2026 by BinarX offering a</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Inherit"/>
+      </rPr>
+      <t xml:space="preserve"> hands-on experience in space science and technology to upper primary students. PAST members worked with Binar to deliver an experience where students built and launched model rockets to learn foundational science and engineering processes.</t>
+    </r>
+  </si>
+  <si>
+    <t>The ADCS integration board was a project to integrate all sensors, actuators, microcontroller and systems required by ADCS, in addition to connectors to interface with other CubeSat subsystems into one board. The completed board allowed development and testing of flight software and the ADCS integration process.</t>
+  </si>
+  <si>
+    <t>The ADCS testbed is a project to develop a housing and actuator system using an air bearing to allow three-axis low-friction movement, providing the capability to test ADCS systems and a full cubesat in a simulated space environment in-house.</t>
+  </si>
+  <si>
+    <t>The detumbling algorithm project produced a stable, robust and effective algorithm to detumble a 1U CubeSat, accounting for real world issues such as sensor noise, perturbations and edge-cases. This algorithm was used in simulations of cubesat pointing control and the space environment to validate and guide CubeSat design choices.</t>
+  </si>
+  <si>
+    <t>./Images/FISH.jpg</t>
+  </si>
+  <si>
+    <t>Ground, Air, Space</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -419,6 +564,17 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="6"/>
+      <color theme="1"/>
+      <name val="Inherit"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Inherit"/>
     </font>
   </fonts>
   <fills count="4">
@@ -468,7 +624,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -477,6 +633,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -811,8 +976,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{009CE143-C523-4CAD-BACF-742F603C1FBF}">
-  <dimension ref="A1:K46"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:K50"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="2" max="2" width="8.6640625" customWidth="1"/>
     <col min="3" max="3" width="36" customWidth="1"/>
@@ -825,7 +990,7 @@
     <col min="11" max="11" width="17.73046875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:11" ht="18">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -860,7 +1025,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11">
       <c r="A2">
         <v>1</v>
       </c>
@@ -889,8 +1054,11 @@
         <v>37</v>
       </c>
       <c r="J2" s="3"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="K2" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
       <c r="A3">
         <v>2</v>
       </c>
@@ -915,9 +1083,15 @@
       <c r="H3" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="J3" s="3"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="I3" t="s">
+        <v>128</v>
+      </c>
+      <c r="J3" s="4"/>
+      <c r="K3" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
       <c r="A4">
         <v>3</v>
       </c>
@@ -942,9 +1116,15 @@
       <c r="H4" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="J4" s="3"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="I4" t="s">
+        <v>129</v>
+      </c>
+      <c r="J4" s="4"/>
+      <c r="K4" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="99.75">
       <c r="A5">
         <v>4</v>
       </c>
@@ -969,9 +1149,17 @@
       <c r="H5" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="J5" s="3"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="I5" t="s">
+        <v>130</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="K5" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="114">
       <c r="A6">
         <v>5</v>
       </c>
@@ -996,9 +1184,17 @@
       <c r="H6" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="J6" s="3"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="I6" t="s">
+        <v>132</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="K6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="85.5">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1012,7 +1208,7 @@
         <v>2025</v>
       </c>
       <c r="E7" s="1">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>7</v>
@@ -1023,9 +1219,17 @@
       <c r="H7" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="J7" s="3"/>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="I7" t="s">
+        <v>133</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="K7" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="128.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1050,9 +1254,17 @@
       <c r="H8" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="J8" s="3"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="I8" t="s">
+        <v>131</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="K8" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1077,9 +1289,15 @@
       <c r="H9" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="J9" s="3"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="I9" t="s">
+        <v>134</v>
+      </c>
+      <c r="J9" s="4"/>
+      <c r="K9" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1104,9 +1322,15 @@
       <c r="H10" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="J10" s="3"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="I10" t="s">
+        <v>135</v>
+      </c>
+      <c r="J10" s="4"/>
+      <c r="K10" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1131,9 +1355,15 @@
       <c r="H11" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="J11" s="3"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="I11" t="s">
+        <v>136</v>
+      </c>
+      <c r="J11" s="4"/>
+      <c r="K11" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1158,9 +1388,15 @@
       <c r="H12" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="J12" s="3"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="I12" t="s">
+        <v>133</v>
+      </c>
+      <c r="J12" s="4"/>
+      <c r="K12" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="71.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1185,9 +1421,17 @@
       <c r="H13" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="J13" s="3"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="I13" t="s">
+        <v>137</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="K13" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1212,9 +1456,15 @@
       <c r="H14" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="J14" s="3"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="I14" t="s">
+        <v>138</v>
+      </c>
+      <c r="J14" s="4"/>
+      <c r="K14" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="99.75">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1239,11 +1489,17 @@
       <c r="H15" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="J15" t="s">
+      <c r="I15" t="s">
+        <v>138</v>
+      </c>
+      <c r="J15" s="4" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="K15" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1266,11 +1522,17 @@
         <v>15</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="J16" s="3"/>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.45">
+        <v>164</v>
+      </c>
+      <c r="I16" t="s">
+        <v>142</v>
+      </c>
+      <c r="J16" s="4"/>
+      <c r="K16" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="114">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1295,11 +1557,17 @@
       <c r="H17" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="J17" t="s">
+      <c r="I17" t="s">
+        <v>141</v>
+      </c>
+      <c r="J17" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="K17" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1324,8 +1592,15 @@
       <c r="H18" s="1" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="I18" t="s">
+        <v>140</v>
+      </c>
+      <c r="J18" s="4"/>
+      <c r="K18" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1350,8 +1625,15 @@
       <c r="H19" s="1" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="I19" t="s">
+        <v>140</v>
+      </c>
+      <c r="J19" s="4"/>
+      <c r="K19" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="99.75">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1376,11 +1658,17 @@
       <c r="H20" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="J20" t="s">
+      <c r="I20" t="s">
+        <v>138</v>
+      </c>
+      <c r="J20" s="4" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="K20" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1405,8 +1693,15 @@
       <c r="H21" s="1" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="I21" t="s">
+        <v>139</v>
+      </c>
+      <c r="J21" s="4"/>
+      <c r="K21" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1431,8 +1726,15 @@
       <c r="H22" s="1" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="I22" t="s">
+        <v>143</v>
+      </c>
+      <c r="J22" s="4"/>
+      <c r="K22" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1457,8 +1759,15 @@
       <c r="H23" s="1" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="I23" t="s">
+        <v>144</v>
+      </c>
+      <c r="J23" s="4"/>
+      <c r="K23" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1483,8 +1792,15 @@
       <c r="H24" s="1" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="I24" t="s">
+        <v>145</v>
+      </c>
+      <c r="J24" s="4"/>
+      <c r="K24" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1509,8 +1825,15 @@
       <c r="H25" s="1" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="I25" t="s">
+        <v>146</v>
+      </c>
+      <c r="J25" s="4"/>
+      <c r="K25" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1535,8 +1858,15 @@
       <c r="H26" s="1" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="I26" t="s">
+        <v>147</v>
+      </c>
+      <c r="J26" s="4"/>
+      <c r="K26" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1561,8 +1891,15 @@
       <c r="H27" s="1" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="I27" t="s">
+        <v>146</v>
+      </c>
+      <c r="J27" s="4"/>
+      <c r="K27" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1587,8 +1924,15 @@
       <c r="H28" s="1" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="I28" t="s">
+        <v>149</v>
+      </c>
+      <c r="J28" s="4"/>
+      <c r="K28" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1613,8 +1957,15 @@
       <c r="H29" s="1" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="I29" t="s">
+        <v>146</v>
+      </c>
+      <c r="J29" s="4"/>
+      <c r="K29" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1639,8 +1990,15 @@
       <c r="H30" s="1" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="I30" t="s">
+        <v>146</v>
+      </c>
+      <c r="J30" s="4"/>
+      <c r="K30" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1665,8 +2023,15 @@
       <c r="H31" s="1" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="I31" t="s">
+        <v>147</v>
+      </c>
+      <c r="J31" s="4"/>
+      <c r="K31" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1691,8 +2056,15 @@
       <c r="H32" s="1" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="I32" t="s">
+        <v>148</v>
+      </c>
+      <c r="J32" s="4"/>
+      <c r="K32" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1717,8 +2089,15 @@
       <c r="H33" s="1" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="I33" t="s">
+        <v>141</v>
+      </c>
+      <c r="J33" s="4"/>
+      <c r="K33" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1743,8 +2122,15 @@
       <c r="H34" s="1" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="I34" t="s">
+        <v>141</v>
+      </c>
+      <c r="J34" s="4"/>
+      <c r="K34" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1769,8 +2155,15 @@
       <c r="H35" s="1" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="I35" t="s">
+        <v>141</v>
+      </c>
+      <c r="J35" s="4"/>
+      <c r="K35" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" ht="57">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1795,8 +2188,17 @@
       <c r="H36" s="1" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="I36" t="s">
+        <v>150</v>
+      </c>
+      <c r="J36" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="K36" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1821,8 +2223,15 @@
       <c r="H37" s="1" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="I37" t="s">
+        <v>151</v>
+      </c>
+      <c r="J37" s="4"/>
+      <c r="K37" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1847,8 +2256,12 @@
       <c r="H38" s="1" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="J38" s="4"/>
+      <c r="K38" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1873,8 +2286,15 @@
       <c r="H39" s="1" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="I39" t="s">
+        <v>152</v>
+      </c>
+      <c r="J39" s="4"/>
+      <c r="K39" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1899,8 +2319,15 @@
       <c r="H40" s="1" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="I40" t="s">
+        <v>153</v>
+      </c>
+      <c r="J40" s="4"/>
+      <c r="K40" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1925,8 +2352,15 @@
       <c r="H41" s="1" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="I41" t="s">
+        <v>141</v>
+      </c>
+      <c r="J41" s="4"/>
+      <c r="K41" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1951,8 +2385,15 @@
       <c r="H42" s="1" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="I42" t="s">
+        <v>154</v>
+      </c>
+      <c r="J42" s="4"/>
+      <c r="K42" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1977,8 +2418,12 @@
       <c r="H43" s="1" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="J43" s="4"/>
+      <c r="K43" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11">
       <c r="A44">
         <v>43</v>
       </c>
@@ -2003,8 +2448,12 @@
       <c r="H44" s="1" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="J44" s="4"/>
+      <c r="K44" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11">
       <c r="A45">
         <v>44</v>
       </c>
@@ -2029,18 +2478,121 @@
       <c r="H45" s="1" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="B46" s="1"/>
-      <c r="D46" s="1"/>
-      <c r="E46" s="1"/>
-      <c r="F46" s="1"/>
-      <c r="G46" s="1"/>
-      <c r="H46" s="1"/>
+      <c r="J45" s="4"/>
+      <c r="K45" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="C46" t="s">
+        <v>121</v>
+      </c>
+      <c r="D46" s="1">
+        <v>2023</v>
+      </c>
+      <c r="E46" s="1">
+        <v>2026</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H46" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="I46" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="J46" s="4"/>
+      <c r="K46" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" ht="138">
+      <c r="A47">
+        <v>45</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C47" t="s">
+        <v>124</v>
+      </c>
+      <c r="D47" s="1">
+        <v>2026</v>
+      </c>
+      <c r="E47" s="1">
+        <v>2026</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H47" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="I47" t="s">
+        <v>127</v>
+      </c>
+      <c r="J47" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="K47" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11">
+      <c r="A48">
+        <v>45</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C48" t="s">
+        <v>126</v>
+      </c>
+      <c r="D48" s="1">
+        <v>2025</v>
+      </c>
+      <c r="E48" s="1">
+        <v>2026</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="G48" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H48" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="I48" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="J48" s="6"/>
+      <c r="K48" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="49" spans="10:10">
+      <c r="J49" s="6"/>
+    </row>
+    <row r="50" spans="10:10">
+      <c r="J50" s="6"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D2:E45">
-    <cfRule type="colorScale" priority="4">
+  <conditionalFormatting sqref="D46:E46">
+    <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -2051,15 +2603,27 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F45">
-    <cfRule type="iconSet" priority="2">
+  <conditionalFormatting sqref="D2:E45 D47:E48">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color theme="5" tint="0.39997558519241921"/>
+        <color theme="4" tint="0.59999389629810485"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F2:F45 F47:F48">
+    <cfRule type="iconSet" priority="8">
       <iconSet>
         <cfvo type="percent" val="0"/>
         <cfvo type="percent" val="33"/>
         <cfvo type="percent" val="67"/>
       </iconSet>
     </cfRule>
-    <cfRule type="colorScale" priority="3">
+    <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -2070,8 +2634,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G45">
-    <cfRule type="iconSet" priority="1">
+  <conditionalFormatting sqref="G2:G45 G47:G48">
+    <cfRule type="iconSet" priority="12">
       <iconSet iconSet="3Symbols2">
         <cfvo type="percent" val="0"/>
         <cfvo type="percent" val="33"/>
@@ -2081,4 +2645,272 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101004AEB57E041483C4788C24AD798662EE0" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d71430372dc1f13b1941cf9619880684">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="4801ea24-2cda-47dd-a258-e252f87d5b95" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ba0ad71eeb0b1d127fbe285f0a4964dd" ns3:_="">
+    <xsd:import namespace="4801ea24-2cda-47dd-a258-e252f87d5b95"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns3:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns3:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns3:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns3:_activity" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceSystemTags" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaLengthInSeconds" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="4801ea24-2cda-47dd-a258-e252f87d5b95" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="_activity" ma:index="11" nillable="true" ma:displayName="_activity" ma:hidden="true" ma:internalName="_activity" ma:readOnly="false">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="12" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="13" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="14" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="15" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSystemTags" ma:index="16" nillable="true" ma:displayName="MediaServiceSystemTags" ma:hidden="true" ma:internalName="MediaServiceSystemTags" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="17" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="18" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="19" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="20" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="21" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="4801ea24-2cda-47dd-a258-e252f87d5b95" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="4801ea24-2cda-47dd-a258-e252f87d5b95" xsi:nil="true"/>
+    <_activity xmlns="4801ea24-2cda-47dd-a258-e252f87d5b95" xsi:nil="true"/>
+    <MigrationWizId xmlns="4801ea24-2cda-47dd-a258-e252f87d5b95" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6CA8792-485F-4A88-9822-C01D85326AB6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="4801ea24-2cda-47dd-a258-e252f87d5b95"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B593FD86-A48A-4A65-B29E-C35D51164D1C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F91F5C1-1C43-483F-B488-33304EA41E97}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4801ea24-2cda-47dd-a258-e252f87d5b95"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
add some more descriptions
</commit_message>
<xml_diff>
--- a/Project List.xlsx
+++ b/Project List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\conno\Documents\UNI\PAST\Project Work\PASTdle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46871AA3-6E55-45C4-93F3-66DCF2EB10A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D214190-B6EE-47A1-B6B5-AAF01E79FE6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{05053F43-13BA-4F95-AF36-FFC7FBE442FD}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="164">
   <si>
     <t>ID</t>
   </si>
@@ -538,9 +538,6 @@
   </si>
   <si>
     <t>The detumbling algorithm project produced a stable, robust and effective algorithm to detumble a 1U CubeSat, accounting for real world issues such as sensor noise, perturbations and edge-cases. This algorithm was used in simulations of cubesat pointing control and the space environment to validate and guide CubeSat design choices.</t>
-  </si>
-  <si>
-    <t>./Images/FISH.jpg</t>
   </si>
   <si>
     <t>Ground, Air, Space</t>
@@ -1054,9 +1051,6 @@
         <v>37</v>
       </c>
       <c r="J2" s="3"/>
-      <c r="K2" t="s">
-        <v>163</v>
-      </c>
     </row>
     <row r="3" spans="1:11">
       <c r="A3">
@@ -1087,9 +1081,6 @@
         <v>128</v>
       </c>
       <c r="J3" s="4"/>
-      <c r="K3" t="s">
-        <v>163</v>
-      </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4">
@@ -1120,9 +1111,6 @@
         <v>129</v>
       </c>
       <c r="J4" s="4"/>
-      <c r="K4" t="s">
-        <v>163</v>
-      </c>
     </row>
     <row r="5" spans="1:11" ht="99.75">
       <c r="A5">
@@ -1155,9 +1143,6 @@
       <c r="J5" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="K5" t="s">
-        <v>163</v>
-      </c>
     </row>
     <row r="6" spans="1:11" ht="114">
       <c r="A6">
@@ -1190,9 +1175,6 @@
       <c r="J6" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="K6" t="s">
-        <v>163</v>
-      </c>
     </row>
     <row r="7" spans="1:11" ht="85.5">
       <c r="A7">
@@ -1225,9 +1207,6 @@
       <c r="J7" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="K7" t="s">
-        <v>163</v>
-      </c>
     </row>
     <row r="8" spans="1:11" ht="128.25">
       <c r="A8">
@@ -1260,9 +1239,6 @@
       <c r="J8" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="K8" t="s">
-        <v>163</v>
-      </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9">
@@ -1293,9 +1269,6 @@
         <v>134</v>
       </c>
       <c r="J9" s="4"/>
-      <c r="K9" t="s">
-        <v>163</v>
-      </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10">
@@ -1326,9 +1299,6 @@
         <v>135</v>
       </c>
       <c r="J10" s="4"/>
-      <c r="K10" t="s">
-        <v>163</v>
-      </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11">
@@ -1359,9 +1329,6 @@
         <v>136</v>
       </c>
       <c r="J11" s="4"/>
-      <c r="K11" t="s">
-        <v>163</v>
-      </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12">
@@ -1392,9 +1359,6 @@
         <v>133</v>
       </c>
       <c r="J12" s="4"/>
-      <c r="K12" t="s">
-        <v>163</v>
-      </c>
     </row>
     <row r="13" spans="1:11" ht="71.25">
       <c r="A13">
@@ -1427,9 +1391,6 @@
       <c r="J13" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="K13" t="s">
-        <v>163</v>
-      </c>
     </row>
     <row r="14" spans="1:11">
       <c r="A14">
@@ -1460,9 +1421,6 @@
         <v>138</v>
       </c>
       <c r="J14" s="4"/>
-      <c r="K14" t="s">
-        <v>163</v>
-      </c>
     </row>
     <row r="15" spans="1:11" ht="99.75">
       <c r="A15">
@@ -1495,9 +1453,6 @@
       <c r="J15" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="K15" t="s">
-        <v>163</v>
-      </c>
     </row>
     <row r="16" spans="1:11">
       <c r="A16">
@@ -1522,17 +1477,14 @@
         <v>15</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="I16" t="s">
         <v>142</v>
       </c>
       <c r="J16" s="4"/>
-      <c r="K16" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" ht="114">
+    </row>
+    <row r="17" spans="1:10" ht="114">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1563,11 +1515,8 @@
       <c r="J17" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="K17" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11">
+    </row>
+    <row r="18" spans="1:10">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1596,11 +1545,8 @@
         <v>140</v>
       </c>
       <c r="J18" s="4"/>
-      <c r="K18" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11">
+    </row>
+    <row r="19" spans="1:10">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1629,11 +1575,8 @@
         <v>140</v>
       </c>
       <c r="J19" s="4"/>
-      <c r="K19" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="99.75">
+    </row>
+    <row r="20" spans="1:10" ht="99.75">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1664,11 +1607,8 @@
       <c r="J20" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="K20" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11">
+    </row>
+    <row r="21" spans="1:10">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1697,11 +1637,8 @@
         <v>139</v>
       </c>
       <c r="J21" s="4"/>
-      <c r="K21" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11">
+    </row>
+    <row r="22" spans="1:10">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1730,11 +1667,8 @@
         <v>143</v>
       </c>
       <c r="J22" s="4"/>
-      <c r="K22" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11">
+    </row>
+    <row r="23" spans="1:10">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1763,11 +1697,8 @@
         <v>144</v>
       </c>
       <c r="J23" s="4"/>
-      <c r="K23" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11">
+    </row>
+    <row r="24" spans="1:10">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1796,11 +1727,8 @@
         <v>145</v>
       </c>
       <c r="J24" s="4"/>
-      <c r="K24" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11">
+    </row>
+    <row r="25" spans="1:10">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1829,11 +1757,8 @@
         <v>146</v>
       </c>
       <c r="J25" s="4"/>
-      <c r="K25" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11">
+    </row>
+    <row r="26" spans="1:10">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1862,11 +1787,8 @@
         <v>147</v>
       </c>
       <c r="J26" s="4"/>
-      <c r="K26" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11">
+    </row>
+    <row r="27" spans="1:10">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1895,11 +1817,8 @@
         <v>146</v>
       </c>
       <c r="J27" s="4"/>
-      <c r="K27" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11">
+    </row>
+    <row r="28" spans="1:10">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1928,11 +1847,8 @@
         <v>149</v>
       </c>
       <c r="J28" s="4"/>
-      <c r="K28" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11">
+    </row>
+    <row r="29" spans="1:10">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1961,11 +1877,8 @@
         <v>146</v>
       </c>
       <c r="J29" s="4"/>
-      <c r="K29" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11">
+    </row>
+    <row r="30" spans="1:10">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1994,11 +1907,8 @@
         <v>146</v>
       </c>
       <c r="J30" s="4"/>
-      <c r="K30" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11">
+    </row>
+    <row r="31" spans="1:10">
       <c r="A31">
         <v>30</v>
       </c>
@@ -2027,11 +1937,8 @@
         <v>147</v>
       </c>
       <c r="J31" s="4"/>
-      <c r="K31" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11">
+    </row>
+    <row r="32" spans="1:10">
       <c r="A32">
         <v>31</v>
       </c>
@@ -2060,11 +1967,8 @@
         <v>148</v>
       </c>
       <c r="J32" s="4"/>
-      <c r="K32" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11">
+    </row>
+    <row r="33" spans="1:10">
       <c r="A33">
         <v>32</v>
       </c>
@@ -2093,11 +1997,8 @@
         <v>141</v>
       </c>
       <c r="J33" s="4"/>
-      <c r="K33" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11">
+    </row>
+    <row r="34" spans="1:10">
       <c r="A34">
         <v>33</v>
       </c>
@@ -2126,11 +2027,8 @@
         <v>141</v>
       </c>
       <c r="J34" s="4"/>
-      <c r="K34" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11">
+    </row>
+    <row r="35" spans="1:10">
       <c r="A35">
         <v>34</v>
       </c>
@@ -2159,11 +2057,8 @@
         <v>141</v>
       </c>
       <c r="J35" s="4"/>
-      <c r="K35" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" ht="57">
+    </row>
+    <row r="36" spans="1:10" ht="57">
       <c r="A36">
         <v>35</v>
       </c>
@@ -2194,11 +2089,8 @@
       <c r="J36" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="K36" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11">
+    </row>
+    <row r="37" spans="1:10">
       <c r="A37">
         <v>36</v>
       </c>
@@ -2227,11 +2119,8 @@
         <v>151</v>
       </c>
       <c r="J37" s="4"/>
-      <c r="K37" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11">
+    </row>
+    <row r="38" spans="1:10">
       <c r="A38">
         <v>37</v>
       </c>
@@ -2257,11 +2146,8 @@
         <v>104</v>
       </c>
       <c r="J38" s="4"/>
-      <c r="K38" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11">
+    </row>
+    <row r="39" spans="1:10">
       <c r="A39">
         <v>38</v>
       </c>
@@ -2290,11 +2176,8 @@
         <v>152</v>
       </c>
       <c r="J39" s="4"/>
-      <c r="K39" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11">
+    </row>
+    <row r="40" spans="1:10">
       <c r="A40">
         <v>39</v>
       </c>
@@ -2323,11 +2206,8 @@
         <v>153</v>
       </c>
       <c r="J40" s="4"/>
-      <c r="K40" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11">
+    </row>
+    <row r="41" spans="1:10">
       <c r="A41">
         <v>40</v>
       </c>
@@ -2356,11 +2236,8 @@
         <v>141</v>
       </c>
       <c r="J41" s="4"/>
-      <c r="K41" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11">
+    </row>
+    <row r="42" spans="1:10">
       <c r="A42">
         <v>41</v>
       </c>
@@ -2389,11 +2266,8 @@
         <v>154</v>
       </c>
       <c r="J42" s="4"/>
-      <c r="K42" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11">
+    </row>
+    <row r="43" spans="1:10">
       <c r="A43">
         <v>42</v>
       </c>
@@ -2419,11 +2293,8 @@
         <v>104</v>
       </c>
       <c r="J43" s="4"/>
-      <c r="K43" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11">
+    </row>
+    <row r="44" spans="1:10">
       <c r="A44">
         <v>43</v>
       </c>
@@ -2449,11 +2320,8 @@
         <v>110</v>
       </c>
       <c r="J44" s="4"/>
-      <c r="K44" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11">
+    </row>
+    <row r="45" spans="1:10">
       <c r="A45">
         <v>44</v>
       </c>
@@ -2479,11 +2347,8 @@
         <v>104</v>
       </c>
       <c r="J45" s="4"/>
-      <c r="K45" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11">
+    </row>
+    <row r="46" spans="1:10">
       <c r="A46">
         <v>45</v>
       </c>
@@ -2512,11 +2377,8 @@
         <v>155</v>
       </c>
       <c r="J46" s="4"/>
-      <c r="K46" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" ht="138">
+    </row>
+    <row r="47" spans="1:10" ht="138">
       <c r="A47">
         <v>45</v>
       </c>
@@ -2547,11 +2409,8 @@
       <c r="J47" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="K47" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11">
+    </row>
+    <row r="48" spans="1:10">
       <c r="A48">
         <v>45</v>
       </c>
@@ -2580,9 +2439,6 @@
         <v>155</v>
       </c>
       <c r="J48" s="6"/>
-      <c r="K48" t="s">
-        <v>163</v>
-      </c>
     </row>
     <row r="49" spans="10:10">
       <c r="J49" s="6"/>

</xml_diff>